<commit_message>
A prova d'inversor: fonts verificades, auditoria del model i Q&A
- Nou 00_EXECUTIVE/Investor Q&A.pdf: 25 preguntes difícils amb respostes
  i taula de verificació de xifres clau.
- _build/audit_model.py: recalcula Base i Optimista amb LibreOffice i
  refà VAN, TIR i repartiment unitari fora del model (9/9 correctes);
  l'Optimista sense valor terminal es mostra explícitament.
- Fonts: creixement de Habanos (+16% companyia / +14,7% Halfwheel),
  12.858 llicències d'expenedoria (2024), abast de les sancions a
  Tabacalera; noves S52–S54. Aranzel 26% i marge 9% marcats PROBABLE.
- Pes de l'Estat unificat al valor del model (41,5%) a tots els documents.
- Dossier (26 pàg.): proposta per trams (pendent de D12) i equip.
- Cua de renders: medalló amb només les mans (sense cara).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Cf1VjW9mqckGqcvuVgoNK
</commit_message>
<xml_diff>
--- a/PROYECTO_CIGARS_CUBA_2027/03_BUSINESS_CASE/Financial Model 2027–2031.xlsx
+++ b/PROYECTO_CIGARS_CUBA_2027/03_BUSINESS_CASE/Financial Model 2027–2031.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1153" uniqueCount="833">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="847">
   <si>
     <t xml:space="preserve">ARNALDO — Modelo financiero 2027–2031 · Dashboard ejecutivo</t>
   </si>
@@ -2230,6 +2230,48 @@
   </si>
   <si>
     <t xml:space="preserve">https://trademark.justia.com/owners/gryson-naamloze-vennootschap-1326237</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Objective — «Los estancos descienden un 3% en diez años» (17/02/2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secundaria (cita datos oficiales)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.858 licencias de expendeduría en 2024 (13.287 en 2015). Otra cifra de 16.049 (prensa, 2023) no es coherente con el resto y no se usa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://theobjective.com/sociedad/2025-02-17/estancos-diez-anos-fumadores-diarios-9/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Halfwheel — Habanos S.A. reports $827 million in revenue for 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirma 827 M USD en 2024; calcula +14,7% frente al +16% que comunica la compañía. Mercados: China, España, Suiza, Reino Unido, Alemania; Europa 54%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://halfwheel.com/habanos-s-a-reports-827-million-in-revenue-for-2024-a-14-7-percent-increase/447655/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diario de Cuba / Cigars-Connect / Nicotine Insider — Tabacalera bajo supervisión del Tesoro tras las sanciones UE a Chen Zhi (ago.–sep. 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secundaria (varias fuentes coincidentes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UE sanciona a Chen Zhi y Prince Holding Group (30/07/2026); Chen Zhi controlaba indirectamente el 57,1% de Allied Cigar; Tabacalera (controla ITI Cigars, 50% de Habanos S.A.) opera con cuentas bloqueadas y necesita autorización del Tesoro para pagar; su CEO comunicó que la empresa está sujeta a las sanciones. Las autoridades no lo han confirmado públicamente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.cigars-connect.com/en/tabacalera-placed-under-spanish-treasury-oversight-following-eu-sanctions-against-chen-zhi/</t>
   </si>
   <si>
     <t xml:space="preserve">N01</t>
@@ -3174,11 +3216,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="92930207"/>
-        <c:axId val="34303184"/>
+        <c:axId val="58275696"/>
+        <c:axId val="40186320"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="92930207"/>
+        <c:axId val="58275696"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3210,7 +3252,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34303184"/>
+        <c:crossAx val="40186320"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3218,7 +3260,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="34303184"/>
+        <c:axId val="40186320"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3260,7 +3302,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92930207"/>
+        <c:crossAx val="58275696"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3551,11 +3593,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="94050562"/>
-        <c:axId val="75697142"/>
+        <c:axId val="55791014"/>
+        <c:axId val="42515356"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="94050562"/>
+        <c:axId val="55791014"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3587,7 +3629,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="75697142"/>
+        <c:crossAx val="42515356"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3595,7 +3637,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="75697142"/>
+        <c:axId val="42515356"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3637,7 +3679,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94050562"/>
+        <c:crossAx val="55791014"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4072,11 +4114,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="20652155"/>
-        <c:axId val="94115888"/>
+        <c:axId val="44290564"/>
+        <c:axId val="41852853"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="20652155"/>
+        <c:axId val="44290564"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4108,7 +4150,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94115888"/>
+        <c:crossAx val="41852853"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4116,7 +4158,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94115888"/>
+        <c:axId val="41852853"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4158,7 +4200,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20652155"/>
+        <c:crossAx val="44290564"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8640,7 +8682,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -9729,19 +9771,19 @@
         <v>737</v>
       </c>
       <c r="C57" s="40" t="s">
-        <v>733</v>
+        <v>508</v>
       </c>
       <c r="D57" s="40" t="s">
         <v>738</v>
       </c>
       <c r="E57" s="40" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="F57" s="40" t="s">
         <v>739</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="40" t="s">
         <v>740</v>
       </c>
@@ -9749,170 +9791,230 @@
         <v>741</v>
       </c>
       <c r="C58" s="40" t="s">
-        <v>733</v>
+        <v>742</v>
       </c>
       <c r="D58" s="40" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="E58" s="40" t="s">
         <v>60</v>
       </c>
       <c r="F58" s="40" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="40" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="B59" s="40" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="C59" s="40" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D59" s="40" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="E59" s="40" t="s">
         <v>60</v>
       </c>
       <c r="F59" s="40" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="40" t="s">
+        <v>750</v>
+      </c>
+      <c r="B60" s="40" t="s">
+        <v>751</v>
+      </c>
+      <c r="C60" s="40" t="s">
         <v>747</v>
       </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="40" t="s">
-        <v>748</v>
-      </c>
-      <c r="B60" s="40" t="s">
-        <v>749</v>
-      </c>
-      <c r="C60" s="40" t="s">
-        <v>733</v>
-      </c>
       <c r="D60" s="40" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="E60" s="40" t="s">
         <v>60</v>
       </c>
       <c r="F60" s="40" t="s">
-        <v>751</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="40" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="B61" s="40" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="C61" s="40" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D61" s="40" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="E61" s="40" t="s">
         <v>60</v>
       </c>
       <c r="F61" s="40" t="s">
-        <v>755</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="40" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="B62" s="40" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="C62" s="40" t="s">
-        <v>733</v>
+        <v>747</v>
       </c>
       <c r="D62" s="40" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="E62" s="40" t="s">
-        <v>759</v>
+        <v>60</v>
       </c>
       <c r="F62" s="40" t="s">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="23" t="s">
         <v>761</v>
       </c>
-      <c r="B64" s="24"/>
-      <c r="C64" s="24"/>
-      <c r="D64" s="24"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="24"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="40" t="s">
+        <v>762</v>
+      </c>
+      <c r="B63" s="40" t="s">
+        <v>763</v>
+      </c>
+      <c r="C63" s="40" t="s">
+        <v>747</v>
+      </c>
+      <c r="D63" s="40" t="s">
+        <v>764</v>
+      </c>
+      <c r="E63" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="F63" s="40" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="40" t="s">
+        <v>766</v>
+      </c>
+      <c r="B64" s="40" t="s">
+        <v>767</v>
+      </c>
+      <c r="C64" s="40" t="s">
+        <v>747</v>
+      </c>
+      <c r="D64" s="40" t="s">
+        <v>768</v>
+      </c>
+      <c r="E64" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="F64" s="40" t="s">
+        <v>769</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="3" t="s">
-        <v>762</v>
-      </c>
-      <c r="B65" s="3"/>
-      <c r="C65" s="3"/>
-      <c r="D65" s="4" t="str">
-        <f aca="false">IF(SUMPRODUCT(ABS(Engine!$C$84:$Y$84))&lt;0.5,"OK","ERROR")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="3" t="s">
-        <v>763</v>
-      </c>
-      <c r="B66" s="3"/>
-      <c r="C66" s="3"/>
-      <c r="D66" s="4" t="str">
-        <f aca="false">IF(ABS('Import &amp; Taxes'!D29-1)&lt;0.0001,"OK","ERROR")</f>
-        <v>OK</v>
+      <c r="A65" s="40" t="s">
+        <v>770</v>
+      </c>
+      <c r="B65" s="40" t="s">
+        <v>771</v>
+      </c>
+      <c r="C65" s="40" t="s">
+        <v>747</v>
+      </c>
+      <c r="D65" s="40" t="s">
+        <v>772</v>
+      </c>
+      <c r="E65" s="40" t="s">
+        <v>773</v>
+      </c>
+      <c r="F65" s="40" t="s">
+        <v>774</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
-        <v>764</v>
-      </c>
-      <c r="B67" s="3"/>
-      <c r="C67" s="3"/>
-      <c r="D67" s="4" t="str">
-        <f aca="false">IF(SUMPRODUCT(ABS('Cash Flow'!B19:F19))&lt;0.5,"OK","ERROR")</f>
-        <v>OK</v>
-      </c>
+      <c r="A67" s="23" t="s">
+        <v>775</v>
+      </c>
+      <c r="B67" s="24"/>
+      <c r="C67" s="24"/>
+      <c r="D67" s="24"/>
+      <c r="E67" s="24"/>
+      <c r="F67" s="24"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>765</v>
+        <v>776</v>
       </c>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
       <c r="D68" s="4" t="str">
-        <f aca="false">IF(ABS('Sensitivity Analysis'!C13)&lt;1,"OK","ERROR")</f>
+        <f aca="false">IF(SUMPRODUCT(ABS(Engine!$C$84:$Y$84))&lt;0.5,"OK","ERROR")</f>
         <v>OK</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>766</v>
+        <v>777</v>
       </c>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
       <c r="D69" s="4" t="str">
+        <f aca="false">IF(ABS('Import &amp; Taxes'!D29-1)&lt;0.0001,"OK","ERROR")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="4" t="str">
+        <f aca="false">IF(SUMPRODUCT(ABS('Cash Flow'!B19:F19))&lt;0.5,"OK","ERROR")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="B71" s="3"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="4" t="str">
+        <f aca="false">IF(ABS('Sensitivity Analysis'!C13)&lt;1,"OK","ERROR")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="B72" s="3"/>
+      <c r="C72" s="3"/>
+      <c r="D72" s="4" t="str">
         <f aca="false">IF(MIN(Engine!$C$16:$Y$16)&gt;=-0.01,"OK","ERROR")</f>
         <v>OK</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A65:C65"/>
-    <mergeCell ref="A66:C66"/>
-    <mergeCell ref="A67:C67"/>
     <mergeCell ref="A68:C68"/>
     <mergeCell ref="A69:C69"/>
+    <mergeCell ref="A70:C70"/>
+    <mergeCell ref="A71:C71"/>
+    <mergeCell ref="A72:C72"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9946,12 +10048,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>767</v>
+        <v>781</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>768</v>
+        <v>782</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10054,7 +10156,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>769</v>
+        <v>783</v>
       </c>
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
@@ -10083,7 +10185,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="33" t="s">
-        <v>770</v>
+        <v>784</v>
       </c>
       <c r="C7" s="43" t="n">
         <f aca="false">Assumptions!$C$8+0</f>
@@ -10168,7 +10270,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="33" t="s">
-        <v>771</v>
+        <v>785</v>
       </c>
       <c r="C8" s="44" t="n">
         <f aca="false">'Sales Forecast'!$B$5</f>
@@ -10253,7 +10355,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="s">
-        <v>772</v>
+        <v>786</v>
       </c>
       <c r="C9" s="43" t="n">
         <f aca="false">IF(C7&lt;Assumptions!$C$49,1,0)</f>
@@ -10338,7 +10440,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
-        <v>773</v>
+        <v>787</v>
       </c>
       <c r="C10" s="45" t="n">
         <f aca="false">1/(1-Assumptions!$C$46)+Assumptions!$C$47</f>
@@ -10423,7 +10525,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="33" t="s">
-        <v>774</v>
+        <v>788</v>
       </c>
       <c r="C11" s="44" t="n">
         <f aca="false">0</f>
@@ -10508,7 +10610,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="s">
-        <v>775</v>
+        <v>789</v>
       </c>
       <c r="C12" s="44" t="n">
         <f aca="false">Assumptions!$C$22/12*'Sales Forecast'!$C$5*C9</f>
@@ -10593,7 +10695,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="33" t="s">
-        <v>776</v>
+        <v>790</v>
       </c>
       <c r="C13" s="44" t="n">
         <f aca="false">IF(C9=1,MAX(0,C8*C10+C12-C11),0)</f>
@@ -10763,7 +10865,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="33" t="s">
-        <v>777</v>
+        <v>791</v>
       </c>
       <c r="C15" s="44" t="n">
         <f aca="false">C14*C10</f>
@@ -10848,7 +10950,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="s">
-        <v>778</v>
+        <v>792</v>
       </c>
       <c r="C16" s="44" t="n">
         <f aca="false">C11+C13-C15</f>
@@ -10933,7 +11035,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>779</v>
+        <v>793</v>
       </c>
       <c r="B18" s="24"/>
       <c r="C18" s="24"/>
@@ -11047,7 +11149,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="33" t="s">
-        <v>780</v>
+        <v>794</v>
       </c>
       <c r="C20" s="46" t="n">
         <f aca="false">Assumptions!$C$40/Assumptions!$C$19</f>
@@ -11217,7 +11319,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="33" t="s">
-        <v>781</v>
+        <v>795</v>
       </c>
       <c r="C22" s="46" t="n">
         <f aca="false">(C20+C21+Assumptions!$C$42+Assumptions!$C$43)*(1+Assumptions!$C$15)</f>
@@ -11387,7 +11489,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="33" t="s">
-        <v>782</v>
+        <v>796</v>
       </c>
       <c r="C24" s="46" t="n">
         <f aca="false">C22+C23+Assumptions!$C$16+Assumptions!$C$44</f>
@@ -11642,7 +11744,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="23" t="s">
-        <v>783</v>
+        <v>797</v>
       </c>
       <c r="B28" s="24"/>
       <c r="C28" s="24"/>
@@ -11671,7 +11773,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="33" t="s">
-        <v>784</v>
+        <v>798</v>
       </c>
       <c r="C29" s="47" t="n">
         <f aca="false">C14*C19</f>
@@ -11841,7 +11943,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="33" t="s">
-        <v>785</v>
+        <v>799</v>
       </c>
       <c r="C31" s="47" t="n">
         <f aca="false">C14*C19*Assumptions!$C$13</f>
@@ -11926,7 +12028,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="33" t="s">
-        <v>786</v>
+        <v>800</v>
       </c>
       <c r="C32" s="47" t="n">
         <f aca="false">C14*C19*Assumptions!$C$45</f>
@@ -12011,7 +12113,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="33" t="s">
-        <v>787</v>
+        <v>801</v>
       </c>
       <c r="C33" s="47" t="n">
         <f aca="false">C30-C31-C32</f>
@@ -12096,7 +12198,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="33" t="s">
-        <v>788</v>
+        <v>802</v>
       </c>
       <c r="C34" s="47" t="n">
         <f aca="false">C15*C25</f>
@@ -12266,7 +12368,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="33" t="s">
-        <v>789</v>
+        <v>803</v>
       </c>
       <c r="C36" s="47" t="n">
         <f aca="false">C15*C24</f>
@@ -12351,7 +12453,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="33" t="s">
-        <v>790</v>
+        <v>804</v>
       </c>
       <c r="C37" s="47" t="n">
         <f aca="false">IF(C13&gt;0,Assumptions!$C$18*Assumptions!$C$17,0)</f>
@@ -12521,7 +12623,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="33" t="s">
-        <v>791</v>
+        <v>805</v>
       </c>
       <c r="C39" s="47" t="n">
         <f aca="false">C35-C36-C37-C38</f>
@@ -12776,7 +12878,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="33" t="s">
-        <v>792</v>
+        <v>806</v>
       </c>
       <c r="C42" s="47" t="n">
         <f aca="false">'Operating Expenses'!$C$22</f>
@@ -12861,7 +12963,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="33" t="s">
-        <v>793</v>
+        <v>807</v>
       </c>
       <c r="C43" s="47" t="n">
         <f aca="false">0+C42</f>
@@ -13031,7 +13133,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="33" t="s">
-        <v>794</v>
+        <v>808</v>
       </c>
       <c r="C45" s="47" t="n">
         <f aca="false">0+C44</f>
@@ -13116,7 +13218,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="33" t="s">
-        <v>795</v>
+        <v>809</v>
       </c>
       <c r="C46" s="47" t="n">
         <f aca="false">C43-C45</f>
@@ -13286,7 +13388,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="33" t="s">
-        <v>796</v>
+        <v>810</v>
       </c>
       <c r="C48" s="47" t="n">
         <f aca="false">0*Assumptions!$C$31</f>
@@ -13456,7 +13558,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="33" t="s">
-        <v>797</v>
+        <v>811</v>
       </c>
       <c r="C50" s="47" t="n">
         <f aca="false">0</f>
@@ -13541,7 +13643,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="33" t="s">
-        <v>798</v>
+        <v>812</v>
       </c>
       <c r="C51" s="47" t="n">
         <f aca="false">MAX(0,C49-C50)</f>
@@ -13626,7 +13728,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="33" t="s">
-        <v>799</v>
+        <v>813</v>
       </c>
       <c r="C52" s="47" t="n">
         <f aca="false">MAX(0,C50-MAX(C49,0))+MAX(-C49,0)</f>
@@ -13881,7 +13983,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="23" t="s">
-        <v>800</v>
+        <v>814</v>
       </c>
       <c r="B56" s="24"/>
       <c r="C56" s="24"/>
@@ -13910,7 +14012,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="33" t="s">
-        <v>801</v>
+        <v>815</v>
       </c>
       <c r="C57" s="47" t="n">
         <f aca="false">C16*C24</f>
@@ -13995,7 +14097,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="33" t="s">
-        <v>802</v>
+        <v>816</v>
       </c>
       <c r="C58" s="47" t="n">
         <f aca="false">IF(Assumptions!$C$26=1,C13,C15)*C25</f>
@@ -14165,7 +14267,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="33" t="s">
-        <v>803</v>
+        <v>817</v>
       </c>
       <c r="C60" s="47" t="n">
         <f aca="false">C33*(1+Assumptions!$C$10)*Assumptions!$C$24/365</f>
@@ -14250,7 +14352,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="33" t="s">
-        <v>804</v>
+        <v>818</v>
       </c>
       <c r="C61" s="47" t="n">
         <f aca="false">Assumptions!$C$23*D13*(D20+D21+Assumptions!$C$42)*MIN(1,Assumptions!$C$48/12)</f>
@@ -14335,7 +14437,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="33" t="s">
-        <v>805</v>
+        <v>819</v>
       </c>
       <c r="C62" s="47" t="n">
         <f aca="false">(C13*(C22+C23)+C58)*Assumptions!$C$10</f>
@@ -14420,7 +14522,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="33" t="s">
-        <v>806</v>
+        <v>820</v>
       </c>
       <c r="C63" s="47" t="n">
         <f aca="false">C62*Assumptions!$C$27</f>
@@ -14505,7 +14607,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="33" t="s">
-        <v>807</v>
+        <v>821</v>
       </c>
       <c r="C64" s="47" t="n">
         <f aca="false">C40*Assumptions!$C$25/365</f>
@@ -14590,7 +14692,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="33" t="s">
-        <v>808</v>
+        <v>822</v>
       </c>
       <c r="C65" s="47" t="n">
         <f aca="false">C33*Assumptions!$C$10</f>
@@ -14675,7 +14777,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="33" t="s">
-        <v>809</v>
+        <v>823</v>
       </c>
       <c r="C66" s="47" t="n">
         <f aca="false">C65*Assumptions!$C$27</f>
@@ -14760,7 +14862,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="34" t="s">
-        <v>810</v>
+        <v>824</v>
       </c>
       <c r="C67" s="47" t="n">
         <f aca="false">C57+C59+C60+C61+C63-C64-C66</f>
@@ -14845,7 +14947,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="33" t="s">
-        <v>811</v>
+        <v>825</v>
       </c>
       <c r="C68" s="47" t="n">
         <f aca="false">C67-0</f>
@@ -14930,7 +15032,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="23" t="s">
-        <v>812</v>
+        <v>826</v>
       </c>
       <c r="B70" s="24"/>
       <c r="C70" s="24"/>
@@ -14959,7 +15061,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="33" t="s">
-        <v>813</v>
+        <v>827</v>
       </c>
       <c r="C71" s="47" t="n">
         <f aca="false">C54+C44-C68</f>
@@ -15044,7 +15146,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="33" t="s">
-        <v>814</v>
+        <v>828</v>
       </c>
       <c r="C72" s="47" t="n">
         <f aca="false">-C42</f>
@@ -15214,7 +15316,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="33" t="s">
-        <v>815</v>
+        <v>829</v>
       </c>
       <c r="C74" s="47" t="n">
         <f aca="false">0-0+C71+C72+C73</f>
@@ -15299,7 +15401,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="33" t="s">
-        <v>816</v>
+        <v>830</v>
       </c>
       <c r="C75" s="47" t="n">
         <f aca="false">MAX(0,Assumptions!$C$32-C74)</f>
@@ -15384,7 +15486,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="33" t="s">
-        <v>817</v>
+        <v>831</v>
       </c>
       <c r="C76" s="47" t="n">
         <f aca="false">C75-0</f>
@@ -15554,7 +15656,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="23" t="s">
-        <v>818</v>
+        <v>832</v>
       </c>
       <c r="B79" s="24"/>
       <c r="C79" s="24"/>
@@ -15583,7 +15685,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="33" t="s">
-        <v>819</v>
+        <v>833</v>
       </c>
       <c r="C80" s="47" t="n">
         <f aca="false">C77+C57+C59+C60+C61+C63+C46</f>
@@ -15668,7 +15770,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="33" t="s">
-        <v>820</v>
+        <v>834</v>
       </c>
       <c r="C81" s="47" t="n">
         <f aca="false">C64+C66+C75</f>
@@ -15838,7 +15940,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="33" t="s">
-        <v>821</v>
+        <v>835</v>
       </c>
       <c r="C83" s="47" t="n">
         <f aca="false">Assumptions!$C$9+C82</f>
@@ -15923,7 +16025,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="34" t="s">
-        <v>822</v>
+        <v>836</v>
       </c>
       <c r="C84" s="48" t="n">
         <f aca="false">ROUND(C80-C81-C83,2)</f>
@@ -16008,7 +16110,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="23" t="s">
-        <v>823</v>
+        <v>837</v>
       </c>
       <c r="B86" s="24"/>
       <c r="C86" s="24"/>
@@ -16037,7 +16139,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="34" t="s">
-        <v>824</v>
+        <v>838</v>
       </c>
       <c r="C87" s="47" t="n">
         <f aca="false">C41-C53-C68-C42</f>
@@ -16207,7 +16309,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="33" t="s">
-        <v>825</v>
+        <v>839</v>
       </c>
       <c r="C89" s="47" t="n">
         <f aca="false">IF(0=4,MAX(0,C41)*Assumptions!$C$35,0)</f>
@@ -16377,7 +16479,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="33" t="s">
-        <v>826</v>
+        <v>840</v>
       </c>
       <c r="C91" s="49" t="n">
         <f aca="false">1/(1+Assumptions!$C$34)^(0+1)</f>
@@ -16547,7 +16649,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="33" t="s">
-        <v>827</v>
+        <v>841</v>
       </c>
       <c r="C93" s="43" t="str">
         <f aca="false">IF(AND(C88&gt;=0,-1&lt;0),C7,"")</f>
@@ -16632,7 +16734,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="33" t="s">
-        <v>828</v>
+        <v>842</v>
       </c>
       <c r="C94" s="47" t="n">
         <f aca="false">C47*(1-Assumptions!$C$30)</f>
@@ -16717,7 +16819,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="33" t="s">
-        <v>829</v>
+        <v>843</v>
       </c>
       <c r="C95" s="47" t="n">
         <f aca="false">C67+C46</f>
@@ -16802,7 +16904,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="33" t="s">
-        <v>830</v>
+        <v>844</v>
       </c>
       <c r="C96" s="50" t="n">
         <f aca="false">IF((C95+0)/2&gt;1000,C94/((C95+0)/2),"n/a")</f>
@@ -16887,7 +16989,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="33" t="s">
-        <v>831</v>
+        <v>845</v>
       </c>
       <c r="C97" s="44" t="str">
         <f aca="false">IF(C26&gt;0,(C40+Assumptions!$C$18*Assumptions!$C$17)/C26,"n/a")</f>
@@ -16972,7 +17074,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="33" t="s">
-        <v>832</v>
+        <v>846</v>
       </c>
       <c r="C98" s="44" t="str">
         <f aca="false">IF(C26&gt;0,(C40+Assumptions!$C$18*Assumptions!$C$17+C44)/C26,"n/a")</f>

</xml_diff>

<commit_message>
Ruta A v3 «Casa cubana clàssica»: fora fulla i chaveta, gramàtica de les cases de Habanos
- Dossier: nova pàgina de direcció creativa amb els codis comuns de les
  cases (signatura, lacre i or amb perlat, cartel·la, retrat, segona
  anella, habilitació de la caixa, cedre amb la marca a foc).
- Fora del dossier les imatges de la fulla i la chaveta; pàgines noves de
  doble anella i caixa quan hi hagi els renders v3.
- Brief d'identitat, pla de negoci i Prompt Pack actualitzats; fonts
  S55–S58 (Bock, glossari Habanos, habilitació de la caixa, Bolívar).
- Cua de renders v3 per a la propera quota.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017Cf1VjW9mqckGqcvuVgoNK
</commit_message>
<xml_diff>
--- a/PROYECTO_CIGARS_CUBA_2027/03_BUSINESS_CASE/Financial Model 2027–2031.xlsx
+++ b/PROYECTO_CIGARS_CUBA_2027/03_BUSINESS_CASE/Financial Model 2027–2031.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="847">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1195" uniqueCount="864">
   <si>
     <t xml:space="preserve">ARNALDO — Modelo financiero 2027–2031 · Dashboard ejecutivo</t>
   </si>
@@ -2257,6 +2257,57 @@
   </si>
   <si>
     <t xml:space="preserve">https://halfwheel.com/habanos-s-a-reports-827-million-in-revenue-for-2024-a-14-7-percent-increase/447655/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wikipedia — Cigar band</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se atribuye a Gustave Bock, fabricante en Cuba en el siglo XIX, la invención de la anilla: anillas de papel con su firma para distinguir sus puros de exportación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://en.wikipedia.org/wiki/Cigar_band</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Habanos S.A. — Glossary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anilla: término cubano para la vitola de papel; habilitaciones: decoraciones de la caja, cada una con su nombre tradicional, aplicadas a mano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.habanos.com/en/glossary/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cohiba Atmosphere — Dressing the cigar box</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secundaria (red de Habanos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vista (imagen superior que celebra la marca), bofetón o filete (hoja protectora decorada), larguero (tira de los lados largos con la marca) y costero (tira de los lados cortos con la vitola).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://cohibaatmosphere.com.my/dressing-the-cigar-box/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cigar Aficionado — Habanos S.A. (ficha de la compañía)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bolívar (creada en 1902): la imagen de su epónimo, Simón Bolívar, forma parte de la marca.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.cigaraficionado.com/company/habanos-s-a</t>
   </si>
   <si>
     <t xml:space="preserve">S54</t>
@@ -3216,11 +3267,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="58275696"/>
-        <c:axId val="40186320"/>
+        <c:axId val="43161995"/>
+        <c:axId val="41402727"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="58275696"/>
+        <c:axId val="43161995"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3252,7 +3303,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40186320"/>
+        <c:crossAx val="41402727"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3260,7 +3311,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40186320"/>
+        <c:axId val="41402727"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3302,7 +3353,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58275696"/>
+        <c:crossAx val="43161995"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3593,11 +3644,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="55791014"/>
-        <c:axId val="42515356"/>
+        <c:axId val="94239966"/>
+        <c:axId val="74305209"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="55791014"/>
+        <c:axId val="94239966"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3629,7 +3680,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42515356"/>
+        <c:crossAx val="74305209"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3637,7 +3688,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42515356"/>
+        <c:axId val="74305209"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3679,7 +3730,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55791014"/>
+        <c:crossAx val="94239966"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4114,11 +4165,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="44290564"/>
-        <c:axId val="41852853"/>
+        <c:axId val="96867540"/>
+        <c:axId val="78779288"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="44290564"/>
+        <c:axId val="96867540"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4150,7 +4201,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41852853"/>
+        <c:crossAx val="78779288"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4158,7 +4209,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41852853"/>
+        <c:axId val="78779288"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4200,7 +4251,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44290564"/>
+        <c:crossAx val="96867540"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8682,7 +8733,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -9783,7 +9834,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="40" t="s">
         <v>740</v>
       </c>
@@ -9791,87 +9842,87 @@
         <v>741</v>
       </c>
       <c r="C58" s="40" t="s">
+        <v>508</v>
+      </c>
+      <c r="D58" s="40" t="s">
         <v>742</v>
-      </c>
-      <c r="D58" s="40" t="s">
-        <v>743</v>
       </c>
       <c r="E58" s="40" t="s">
         <v>60</v>
       </c>
       <c r="F58" s="40" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="40" t="s">
+        <v>744</v>
+      </c>
+      <c r="B59" s="40" t="s">
         <v>745</v>
       </c>
-      <c r="B59" s="40" t="s">
+      <c r="C59" s="40" t="s">
+        <v>614</v>
+      </c>
+      <c r="D59" s="40" t="s">
         <v>746</v>
       </c>
-      <c r="C59" s="40" t="s">
+      <c r="E59" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="F59" s="40" t="s">
         <v>747</v>
-      </c>
-      <c r="D59" s="40" t="s">
-        <v>748</v>
-      </c>
-      <c r="E59" s="40" t="s">
-        <v>60</v>
-      </c>
-      <c r="F59" s="40" t="s">
-        <v>749</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="40" t="s">
+        <v>748</v>
+      </c>
+      <c r="B60" s="40" t="s">
+        <v>749</v>
+      </c>
+      <c r="C60" s="40" t="s">
         <v>750</v>
       </c>
-      <c r="B60" s="40" t="s">
+      <c r="D60" s="40" t="s">
         <v>751</v>
-      </c>
-      <c r="C60" s="40" t="s">
-        <v>747</v>
-      </c>
-      <c r="D60" s="40" t="s">
-        <v>752</v>
       </c>
       <c r="E60" s="40" t="s">
         <v>60</v>
       </c>
       <c r="F60" s="40" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="40" t="s">
         <v>753</v>
       </c>
-    </row>
-    <row r="61" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="40" t="s">
+      <c r="B61" s="40" t="s">
         <v>754</v>
       </c>
-      <c r="B61" s="40" t="s">
+      <c r="C61" s="40" t="s">
+        <v>508</v>
+      </c>
+      <c r="D61" s="40" t="s">
         <v>755</v>
-      </c>
-      <c r="C61" s="40" t="s">
-        <v>747</v>
-      </c>
-      <c r="D61" s="40" t="s">
-        <v>756</v>
       </c>
       <c r="E61" s="40" t="s">
         <v>60</v>
       </c>
       <c r="F61" s="40" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="40" t="s">
         <v>757</v>
       </c>
-    </row>
-    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="40" t="s">
+      <c r="B62" s="40" t="s">
         <v>758</v>
       </c>
-      <c r="B62" s="40" t="s">
+      <c r="C62" s="40" t="s">
         <v>759</v>
-      </c>
-      <c r="C62" s="40" t="s">
-        <v>747</v>
       </c>
       <c r="D62" s="40" t="s">
         <v>760</v>
@@ -9883,7 +9934,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="40" t="s">
         <v>762</v>
       </c>
@@ -9891,130 +9942,210 @@
         <v>763</v>
       </c>
       <c r="C63" s="40" t="s">
-        <v>747</v>
+        <v>764</v>
       </c>
       <c r="D63" s="40" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="E63" s="40" t="s">
         <v>60</v>
       </c>
       <c r="F63" s="40" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="40" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="B64" s="40" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="C64" s="40" t="s">
-        <v>747</v>
+        <v>764</v>
       </c>
       <c r="D64" s="40" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="E64" s="40" t="s">
         <v>60</v>
       </c>
       <c r="F64" s="40" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="40" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="B65" s="40" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="C65" s="40" t="s">
-        <v>747</v>
+        <v>764</v>
       </c>
       <c r="D65" s="40" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="E65" s="40" t="s">
-        <v>773</v>
+        <v>60</v>
       </c>
       <c r="F65" s="40" t="s">
         <v>774</v>
       </c>
     </row>
+    <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="40" t="s">
+        <v>775</v>
+      </c>
+      <c r="B66" s="40" t="s">
+        <v>776</v>
+      </c>
+      <c r="C66" s="40" t="s">
+        <v>764</v>
+      </c>
+      <c r="D66" s="40" t="s">
+        <v>777</v>
+      </c>
+      <c r="E66" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="F66" s="40" t="s">
+        <v>778</v>
+      </c>
+    </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="23" t="s">
-        <v>775</v>
-      </c>
-      <c r="B67" s="24"/>
-      <c r="C67" s="24"/>
-      <c r="D67" s="24"/>
-      <c r="E67" s="24"/>
-      <c r="F67" s="24"/>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="3" t="s">
-        <v>776</v>
-      </c>
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="D68" s="4" t="str">
-        <f aca="false">IF(SUMPRODUCT(ABS(Engine!$C$84:$Y$84))&lt;0.5,"OK","ERROR")</f>
-        <v>OK</v>
+      <c r="A67" s="40" t="s">
+        <v>779</v>
+      </c>
+      <c r="B67" s="40" t="s">
+        <v>780</v>
+      </c>
+      <c r="C67" s="40" t="s">
+        <v>764</v>
+      </c>
+      <c r="D67" s="40" t="s">
+        <v>781</v>
+      </c>
+      <c r="E67" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="F67" s="40" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="40" t="s">
+        <v>783</v>
+      </c>
+      <c r="B68" s="40" t="s">
+        <v>784</v>
+      </c>
+      <c r="C68" s="40" t="s">
+        <v>764</v>
+      </c>
+      <c r="D68" s="40" t="s">
+        <v>785</v>
+      </c>
+      <c r="E68" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="F68" s="40" t="s">
+        <v>786</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="3" t="s">
-        <v>777</v>
-      </c>
-      <c r="B69" s="3"/>
-      <c r="C69" s="3"/>
-      <c r="D69" s="4" t="str">
-        <f aca="false">IF(ABS('Import &amp; Taxes'!D29-1)&lt;0.0001,"OK","ERROR")</f>
-        <v>OK</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="3" t="s">
-        <v>778</v>
-      </c>
-      <c r="B70" s="3"/>
-      <c r="C70" s="3"/>
-      <c r="D70" s="4" t="str">
-        <f aca="false">IF(SUMPRODUCT(ABS('Cash Flow'!B19:F19))&lt;0.5,"OK","ERROR")</f>
-        <v>OK</v>
+      <c r="A69" s="40" t="s">
+        <v>787</v>
+      </c>
+      <c r="B69" s="40" t="s">
+        <v>788</v>
+      </c>
+      <c r="C69" s="40" t="s">
+        <v>764</v>
+      </c>
+      <c r="D69" s="40" t="s">
+        <v>789</v>
+      </c>
+      <c r="E69" s="40" t="s">
+        <v>790</v>
+      </c>
+      <c r="F69" s="40" t="s">
+        <v>791</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="3" t="s">
-        <v>779</v>
-      </c>
-      <c r="B71" s="3"/>
-      <c r="C71" s="3"/>
-      <c r="D71" s="4" t="str">
-        <f aca="false">IF(ABS('Sensitivity Analysis'!C13)&lt;1,"OK","ERROR")</f>
-        <v>OK</v>
-      </c>
+      <c r="A71" s="23" t="s">
+        <v>792</v>
+      </c>
+      <c r="B71" s="24"/>
+      <c r="C71" s="24"/>
+      <c r="D71" s="24"/>
+      <c r="E71" s="24"/>
+      <c r="F71" s="24"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>780</v>
+        <v>793</v>
       </c>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
       <c r="D72" s="4" t="str">
+        <f aca="false">IF(SUMPRODUCT(ABS(Engine!$C$84:$Y$84))&lt;0.5,"OK","ERROR")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="B73" s="3"/>
+      <c r="C73" s="3"/>
+      <c r="D73" s="4" t="str">
+        <f aca="false">IF(ABS('Import &amp; Taxes'!D29-1)&lt;0.0001,"OK","ERROR")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="3" t="s">
+        <v>795</v>
+      </c>
+      <c r="B74" s="3"/>
+      <c r="C74" s="3"/>
+      <c r="D74" s="4" t="str">
+        <f aca="false">IF(SUMPRODUCT(ABS('Cash Flow'!B19:F19))&lt;0.5,"OK","ERROR")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="3" t="s">
+        <v>796</v>
+      </c>
+      <c r="B75" s="3"/>
+      <c r="C75" s="3"/>
+      <c r="D75" s="4" t="str">
+        <f aca="false">IF(ABS('Sensitivity Analysis'!C13)&lt;1,"OK","ERROR")</f>
+        <v>OK</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="3" t="s">
+        <v>797</v>
+      </c>
+      <c r="B76" s="3"/>
+      <c r="C76" s="3"/>
+      <c r="D76" s="4" t="str">
         <f aca="false">IF(MIN(Engine!$C$16:$Y$16)&gt;=-0.01,"OK","ERROR")</f>
         <v>OK</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A68:C68"/>
-    <mergeCell ref="A69:C69"/>
-    <mergeCell ref="A70:C70"/>
-    <mergeCell ref="A71:C71"/>
     <mergeCell ref="A72:C72"/>
+    <mergeCell ref="A73:C73"/>
+    <mergeCell ref="A74:C74"/>
+    <mergeCell ref="A75:C75"/>
+    <mergeCell ref="A76:C76"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -10048,12 +10179,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>781</v>
+        <v>798</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>782</v>
+        <v>799</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10156,7 +10287,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>783</v>
+        <v>800</v>
       </c>
       <c r="B6" s="24"/>
       <c r="C6" s="24"/>
@@ -10185,7 +10316,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="33" t="s">
-        <v>784</v>
+        <v>801</v>
       </c>
       <c r="C7" s="43" t="n">
         <f aca="false">Assumptions!$C$8+0</f>
@@ -10270,7 +10401,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="33" t="s">
-        <v>785</v>
+        <v>802</v>
       </c>
       <c r="C8" s="44" t="n">
         <f aca="false">'Sales Forecast'!$B$5</f>
@@ -10355,7 +10486,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="s">
-        <v>786</v>
+        <v>803</v>
       </c>
       <c r="C9" s="43" t="n">
         <f aca="false">IF(C7&lt;Assumptions!$C$49,1,0)</f>
@@ -10440,7 +10571,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="33" t="s">
-        <v>787</v>
+        <v>804</v>
       </c>
       <c r="C10" s="45" t="n">
         <f aca="false">1/(1-Assumptions!$C$46)+Assumptions!$C$47</f>
@@ -10525,7 +10656,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="33" t="s">
-        <v>788</v>
+        <v>805</v>
       </c>
       <c r="C11" s="44" t="n">
         <f aca="false">0</f>
@@ -10610,7 +10741,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="33" t="s">
-        <v>789</v>
+        <v>806</v>
       </c>
       <c r="C12" s="44" t="n">
         <f aca="false">Assumptions!$C$22/12*'Sales Forecast'!$C$5*C9</f>
@@ -10695,7 +10826,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="33" t="s">
-        <v>790</v>
+        <v>807</v>
       </c>
       <c r="C13" s="44" t="n">
         <f aca="false">IF(C9=1,MAX(0,C8*C10+C12-C11),0)</f>
@@ -10865,7 +10996,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="33" t="s">
-        <v>791</v>
+        <v>808</v>
       </c>
       <c r="C15" s="44" t="n">
         <f aca="false">C14*C10</f>
@@ -10950,7 +11081,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="33" t="s">
-        <v>792</v>
+        <v>809</v>
       </c>
       <c r="C16" s="44" t="n">
         <f aca="false">C11+C13-C15</f>
@@ -11035,7 +11166,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>793</v>
+        <v>810</v>
       </c>
       <c r="B18" s="24"/>
       <c r="C18" s="24"/>
@@ -11149,7 +11280,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="33" t="s">
-        <v>794</v>
+        <v>811</v>
       </c>
       <c r="C20" s="46" t="n">
         <f aca="false">Assumptions!$C$40/Assumptions!$C$19</f>
@@ -11319,7 +11450,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="33" t="s">
-        <v>795</v>
+        <v>812</v>
       </c>
       <c r="C22" s="46" t="n">
         <f aca="false">(C20+C21+Assumptions!$C$42+Assumptions!$C$43)*(1+Assumptions!$C$15)</f>
@@ -11489,7 +11620,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="33" t="s">
-        <v>796</v>
+        <v>813</v>
       </c>
       <c r="C24" s="46" t="n">
         <f aca="false">C22+C23+Assumptions!$C$16+Assumptions!$C$44</f>
@@ -11744,7 +11875,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="23" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="B28" s="24"/>
       <c r="C28" s="24"/>
@@ -11773,7 +11904,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="33" t="s">
-        <v>798</v>
+        <v>815</v>
       </c>
       <c r="C29" s="47" t="n">
         <f aca="false">C14*C19</f>
@@ -11943,7 +12074,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="33" t="s">
-        <v>799</v>
+        <v>816</v>
       </c>
       <c r="C31" s="47" t="n">
         <f aca="false">C14*C19*Assumptions!$C$13</f>
@@ -12028,7 +12159,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="33" t="s">
-        <v>800</v>
+        <v>817</v>
       </c>
       <c r="C32" s="47" t="n">
         <f aca="false">C14*C19*Assumptions!$C$45</f>
@@ -12113,7 +12244,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="33" t="s">
-        <v>801</v>
+        <v>818</v>
       </c>
       <c r="C33" s="47" t="n">
         <f aca="false">C30-C31-C32</f>
@@ -12198,7 +12329,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="33" t="s">
-        <v>802</v>
+        <v>819</v>
       </c>
       <c r="C34" s="47" t="n">
         <f aca="false">C15*C25</f>
@@ -12368,7 +12499,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="33" t="s">
-        <v>803</v>
+        <v>820</v>
       </c>
       <c r="C36" s="47" t="n">
         <f aca="false">C15*C24</f>
@@ -12453,7 +12584,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="33" t="s">
-        <v>804</v>
+        <v>821</v>
       </c>
       <c r="C37" s="47" t="n">
         <f aca="false">IF(C13&gt;0,Assumptions!$C$18*Assumptions!$C$17,0)</f>
@@ -12623,7 +12754,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="33" t="s">
-        <v>805</v>
+        <v>822</v>
       </c>
       <c r="C39" s="47" t="n">
         <f aca="false">C35-C36-C37-C38</f>
@@ -12878,7 +13009,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="33" t="s">
-        <v>806</v>
+        <v>823</v>
       </c>
       <c r="C42" s="47" t="n">
         <f aca="false">'Operating Expenses'!$C$22</f>
@@ -12963,7 +13094,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="33" t="s">
-        <v>807</v>
+        <v>824</v>
       </c>
       <c r="C43" s="47" t="n">
         <f aca="false">0+C42</f>
@@ -13133,7 +13264,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="33" t="s">
-        <v>808</v>
+        <v>825</v>
       </c>
       <c r="C45" s="47" t="n">
         <f aca="false">0+C44</f>
@@ -13218,7 +13349,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="33" t="s">
-        <v>809</v>
+        <v>826</v>
       </c>
       <c r="C46" s="47" t="n">
         <f aca="false">C43-C45</f>
@@ -13388,7 +13519,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="33" t="s">
-        <v>810</v>
+        <v>827</v>
       </c>
       <c r="C48" s="47" t="n">
         <f aca="false">0*Assumptions!$C$31</f>
@@ -13558,7 +13689,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="33" t="s">
-        <v>811</v>
+        <v>828</v>
       </c>
       <c r="C50" s="47" t="n">
         <f aca="false">0</f>
@@ -13643,7 +13774,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="33" t="s">
-        <v>812</v>
+        <v>829</v>
       </c>
       <c r="C51" s="47" t="n">
         <f aca="false">MAX(0,C49-C50)</f>
@@ -13728,7 +13859,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="33" t="s">
-        <v>813</v>
+        <v>830</v>
       </c>
       <c r="C52" s="47" t="n">
         <f aca="false">MAX(0,C50-MAX(C49,0))+MAX(-C49,0)</f>
@@ -13983,7 +14114,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="23" t="s">
-        <v>814</v>
+        <v>831</v>
       </c>
       <c r="B56" s="24"/>
       <c r="C56" s="24"/>
@@ -14012,7 +14143,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="33" t="s">
-        <v>815</v>
+        <v>832</v>
       </c>
       <c r="C57" s="47" t="n">
         <f aca="false">C16*C24</f>
@@ -14097,7 +14228,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="33" t="s">
-        <v>816</v>
+        <v>833</v>
       </c>
       <c r="C58" s="47" t="n">
         <f aca="false">IF(Assumptions!$C$26=1,C13,C15)*C25</f>
@@ -14267,7 +14398,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="33" t="s">
-        <v>817</v>
+        <v>834</v>
       </c>
       <c r="C60" s="47" t="n">
         <f aca="false">C33*(1+Assumptions!$C$10)*Assumptions!$C$24/365</f>
@@ -14352,7 +14483,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="33" t="s">
-        <v>818</v>
+        <v>835</v>
       </c>
       <c r="C61" s="47" t="n">
         <f aca="false">Assumptions!$C$23*D13*(D20+D21+Assumptions!$C$42)*MIN(1,Assumptions!$C$48/12)</f>
@@ -14437,7 +14568,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="33" t="s">
-        <v>819</v>
+        <v>836</v>
       </c>
       <c r="C62" s="47" t="n">
         <f aca="false">(C13*(C22+C23)+C58)*Assumptions!$C$10</f>
@@ -14522,7 +14653,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="33" t="s">
-        <v>820</v>
+        <v>837</v>
       </c>
       <c r="C63" s="47" t="n">
         <f aca="false">C62*Assumptions!$C$27</f>
@@ -14607,7 +14738,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="33" t="s">
-        <v>821</v>
+        <v>838</v>
       </c>
       <c r="C64" s="47" t="n">
         <f aca="false">C40*Assumptions!$C$25/365</f>
@@ -14692,7 +14823,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="33" t="s">
-        <v>822</v>
+        <v>839</v>
       </c>
       <c r="C65" s="47" t="n">
         <f aca="false">C33*Assumptions!$C$10</f>
@@ -14777,7 +14908,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="33" t="s">
-        <v>823</v>
+        <v>840</v>
       </c>
       <c r="C66" s="47" t="n">
         <f aca="false">C65*Assumptions!$C$27</f>
@@ -14862,7 +14993,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="34" t="s">
-        <v>824</v>
+        <v>841</v>
       </c>
       <c r="C67" s="47" t="n">
         <f aca="false">C57+C59+C60+C61+C63-C64-C66</f>
@@ -14947,7 +15078,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="33" t="s">
-        <v>825</v>
+        <v>842</v>
       </c>
       <c r="C68" s="47" t="n">
         <f aca="false">C67-0</f>
@@ -15032,7 +15163,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="23" t="s">
-        <v>826</v>
+        <v>843</v>
       </c>
       <c r="B70" s="24"/>
       <c r="C70" s="24"/>
@@ -15061,7 +15192,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="33" t="s">
-        <v>827</v>
+        <v>844</v>
       </c>
       <c r="C71" s="47" t="n">
         <f aca="false">C54+C44-C68</f>
@@ -15146,7 +15277,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="33" t="s">
-        <v>828</v>
+        <v>845</v>
       </c>
       <c r="C72" s="47" t="n">
         <f aca="false">-C42</f>
@@ -15316,7 +15447,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="33" t="s">
-        <v>829</v>
+        <v>846</v>
       </c>
       <c r="C74" s="47" t="n">
         <f aca="false">0-0+C71+C72+C73</f>
@@ -15401,7 +15532,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="33" t="s">
-        <v>830</v>
+        <v>847</v>
       </c>
       <c r="C75" s="47" t="n">
         <f aca="false">MAX(0,Assumptions!$C$32-C74)</f>
@@ -15486,7 +15617,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="33" t="s">
-        <v>831</v>
+        <v>848</v>
       </c>
       <c r="C76" s="47" t="n">
         <f aca="false">C75-0</f>
@@ -15656,7 +15787,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="23" t="s">
-        <v>832</v>
+        <v>849</v>
       </c>
       <c r="B79" s="24"/>
       <c r="C79" s="24"/>
@@ -15685,7 +15816,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="33" t="s">
-        <v>833</v>
+        <v>850</v>
       </c>
       <c r="C80" s="47" t="n">
         <f aca="false">C77+C57+C59+C60+C61+C63+C46</f>
@@ -15770,7 +15901,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="33" t="s">
-        <v>834</v>
+        <v>851</v>
       </c>
       <c r="C81" s="47" t="n">
         <f aca="false">C64+C66+C75</f>
@@ -15940,7 +16071,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="33" t="s">
-        <v>835</v>
+        <v>852</v>
       </c>
       <c r="C83" s="47" t="n">
         <f aca="false">Assumptions!$C$9+C82</f>
@@ -16025,7 +16156,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="34" t="s">
-        <v>836</v>
+        <v>853</v>
       </c>
       <c r="C84" s="48" t="n">
         <f aca="false">ROUND(C80-C81-C83,2)</f>
@@ -16110,7 +16241,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="23" t="s">
-        <v>837</v>
+        <v>854</v>
       </c>
       <c r="B86" s="24"/>
       <c r="C86" s="24"/>
@@ -16139,7 +16270,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="34" t="s">
-        <v>838</v>
+        <v>855</v>
       </c>
       <c r="C87" s="47" t="n">
         <f aca="false">C41-C53-C68-C42</f>
@@ -16309,7 +16440,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="33" t="s">
-        <v>839</v>
+        <v>856</v>
       </c>
       <c r="C89" s="47" t="n">
         <f aca="false">IF(0=4,MAX(0,C41)*Assumptions!$C$35,0)</f>
@@ -16479,7 +16610,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="33" t="s">
-        <v>840</v>
+        <v>857</v>
       </c>
       <c r="C91" s="49" t="n">
         <f aca="false">1/(1+Assumptions!$C$34)^(0+1)</f>
@@ -16649,7 +16780,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="33" t="s">
-        <v>841</v>
+        <v>858</v>
       </c>
       <c r="C93" s="43" t="str">
         <f aca="false">IF(AND(C88&gt;=0,-1&lt;0),C7,"")</f>
@@ -16734,7 +16865,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="33" t="s">
-        <v>842</v>
+        <v>859</v>
       </c>
       <c r="C94" s="47" t="n">
         <f aca="false">C47*(1-Assumptions!$C$30)</f>
@@ -16819,7 +16950,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="33" t="s">
-        <v>843</v>
+        <v>860</v>
       </c>
       <c r="C95" s="47" t="n">
         <f aca="false">C67+C46</f>
@@ -16904,7 +17035,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="33" t="s">
-        <v>844</v>
+        <v>861</v>
       </c>
       <c r="C96" s="50" t="n">
         <f aca="false">IF((C95+0)/2&gt;1000,C94/((C95+0)/2),"n/a")</f>
@@ -16989,7 +17120,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="33" t="s">
-        <v>845</v>
+        <v>862</v>
       </c>
       <c r="C97" s="44" t="str">
         <f aca="false">IF(C26&gt;0,(C40+Assumptions!$C$18*Assumptions!$C$17)/C26,"n/a")</f>
@@ -17074,7 +17205,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="33" t="s">
-        <v>846</v>
+        <v>863</v>
       </c>
       <c r="C98" s="44" t="str">
         <f aca="false">IF(C26&gt;0,(C40+Assumptions!$C$18*Assumptions!$C$17+C44)/C26,"n/a")</f>

</xml_diff>